<commit_message>
docs: update official PhD candidate Le Phuc Hai, advisor Dr. Phung Minh Tuan, and TDTU across all artifacts
</commit_message>
<xml_diff>
--- a/BANG_THEO_DOI_TIEN_DO_LUAN_AN_VA_BAI_BAO.xlsx
+++ b/BANG_THEO_DOI_TIEN_DO_LUAN_AN_VA_BAI_BAO.xlsx
@@ -729,7 +729,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>[Họ và tên Nghiên cứu sinh]</t>
+          <t>Lê Phúc Hải</t>
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>[Mã số NCS]</t>
+          <t>262901002 (Lớp: 26290101)</t>
         </is>
       </c>
       <c r="F5" s="6" t="n"/>
@@ -754,7 +754,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>[Họ hàm, học vị, Họ tên GVHD]</t>
+          <t>TS. Phùng Minh Tuấn</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Viện Đào tạo Sau Đại học / Trường Đại học</t>
+          <t>Trường Đại học Tôn Đức Thắng (TDTU)</t>
         </is>
       </c>
       <c r="F6" s="6" t="n"/>
@@ -779,7 +779,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Marketing &amp; Quản trị Kinh doanh</t>
+          <t>Quản trị kinh doanh</t>
         </is>
       </c>
       <c r="C7" s="6" t="n"/>
@@ -790,7 +790,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>9340101 / 9340115</t>
+          <t>9340101</t>
         </is>
       </c>
       <c r="F7" s="6" t="n"/>
@@ -838,7 +838,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>[Số Quyết định / Ngày ban hành]</t>
+          <t>[Quyết định giao đề tài]</t>
         </is>
       </c>
       <c r="C10" s="6" t="n"/>

</xml_diff>

<commit_message>
feat: recalibrate PhD timeline to 36 months (10/2027 - 10/2030) and ground publications in verified literature
</commit_message>
<xml_diff>
--- a/BANG_THEO_DOI_TIEN_DO_LUAN_AN_VA_BAI_BAO.xlsx
+++ b/BANG_THEO_DOI_TIEN_DO_LUAN_AN_VA_BAI_BAO.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,7 +33,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -73,20 +73,26 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00155724"/>
-      <sz val="11"/>
+      <color rgb="00004085"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00856404"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00004085"/>
-      <sz val="11"/>
+      <color rgb="00486581"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00155724"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -100,8 +106,7 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00155724"/>
+      <color rgb="00627D98"/>
       <sz val="9"/>
     </font>
     <font>
@@ -109,17 +114,6 @@
       <b val="1"/>
       <color rgb="00856404"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="00627D98"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -136,6 +130,18 @@
       <b val="1"/>
       <color rgb="000B69A3"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00155724"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -171,8 +177,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-        <bgColor rgb="00D4EDDA"/>
+        <fgColor rgb="00CCE5FF"/>
+        <bgColor rgb="00CCE5FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -183,20 +189,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCE5FF"/>
-        <bgColor rgb="00CCE5FF"/>
+        <fgColor rgb="00F8F9FA"/>
+        <bgColor rgb="00F8F9FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+        <bgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDF2F7"/>
         <bgColor rgb="00EDF2F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8F9FA"/>
-        <bgColor rgb="00F8F9FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -265,10 +271,13 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -277,49 +286,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -687,29 +693,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HỆ THỐNG THEO DÕI TIẾN ĐỘ LUẬN ÁN TIẾN SĨ &amp; CÔNG BỐ BÀI BÁO QUỐC TẾ</t>
+          <t>HỆ THỐNG THEO DÕI TIẾN ĐỘ LUẬN ÁN TIẾN SĨ &amp; CÔNG BỐ QUỐC TẾ (LỘ TRÌNH 36 THÁNG)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Chuyên ngành: Marketing &amp; Quản trị Kinh doanh | Mục tiêu: 01 Bài WoS (SSCI/SCIE) + 01 Bài Scopus (Q1/Q2)</t>
+          <t>Khóa đào tạo: Tháng 10/2027 – Tháng 10/2030 (36 tháng) | Đơn vị: Trường Đại học Tôn Đức Thắng (TDTU)</t>
         </is>
       </c>
     </row>
@@ -760,7 +766,7 @@
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Đơn vị đào tạo:</t>
+          <t>Cơ sở đào tạo:</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -833,23 +839,23 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Quyết định giao đề tài:</t>
+          <t>Thời gian đào tạo chuẩn:</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>[Quyết định giao đề tài]</t>
+          <t>36 tháng (Bắt đầu: Tháng 10/2027)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Thời hạn bảo vệ:</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Năm 2026 - 2027</t>
+          <t>Thời hạn bảo vệ dự kiến:</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Tháng 10/2030</t>
         </is>
       </c>
       <c r="F10" s="6" t="n"/>
@@ -859,31 +865,31 @@
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>BẢNG ĐIỀU KHIỂN CHỈ SỐ TIẾN ĐỘ TỔNG THỂ (DASHBOARD KPIs)</t>
+          <t>BẢNG ĐIỀU KHIỂN CHỈ SỐ TIẾN ĐỘ 3 NĂM (DASHBOARD KPIs: 2027 - 2030)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>ĐỀ CƯƠNG CHI TIẾT</t>
+          <t>NĂM 1 (10/2027 - 09/2028)</t>
         </is>
       </c>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>5 CHƯƠNG LUẬN ÁN</t>
+          <t>NĂM 2 (10/2028 - 09/2029)</t>
         </is>
       </c>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>BÀI BÁO WOS (Q1/Q2)</t>
+          <t>NĂM 3 (10/2029 - 10/2030)</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>BÀI BÁO SCOPUS (Q1/Q2)</t>
+          <t>TỔNG TIẾN ĐỘ CHUẨN BỊ</t>
         </is>
       </c>
       <c r="G13" s="6" t="n"/>
@@ -891,24 +897,24 @@
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>HOÀN THÀNH (100%)</t>
+          <t>ĐỀ CƯƠNG &amp; PILOT (35%)</t>
         </is>
       </c>
       <c r="B14" s="6" t="n"/>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>ĐANG THỰC HIỆN (35%)</t>
+          <t>KHẢO SÁT &amp; NỘP BÁO (40%)</t>
         </is>
       </c>
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>ĐANG CHUẨN BỊ (25%)</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>ĐANG CHUẨN BỊ (25%)</t>
+          <t>XUẤT BẢN &amp; BẢO VỆ (25%)</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>SẴN SÀNG (ĐÃ CÓ ĐỀ CƯƠNG)</t>
         </is>
       </c>
       <c r="G14" s="6" t="n"/>
@@ -917,464 +923,534 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>DANH MỤC CÁC MỐC TIẾN ĐỘ NGHIÊN CỨU CHÍNH (MILESTONES)</t>
+          <t>LỘ TRÌNH 14 MỐC NGHIÊN CỨU &amp; XUẤT BẢN CHI TIẾT (36 THÁNG: 10/2027 - 10/2030)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Mốc tiến độ nghiên cứu</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Giai đoạn &amp; Mốc tiến độ</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Sản phẩm đầu ra</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Thời hạn mục tiêu</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Thời hạn chuẩn (36 tháng)</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>Tiến độ %</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Trạng thái</t>
         </is>
       </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>Ghi chú thực hiện</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="14" t="n">
+      <c r="A18" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B18" s="15" t="inlineStr">
-        <is>
-          <t>Xây dựng Đề cương nghiên cứu chi tiết &amp; Mô hình</t>
-        </is>
-      </c>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>Đề cương hoàn chỉnh + Sơ đồ SEM</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 10/2026</t>
-        </is>
-      </c>
-      <c r="E18" s="16" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="F18" s="17" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="G18" s="15" t="inlineStr">
-        <is>
-          <t>Đã lập xong file de_cuong_nghien_cuu_chi_tiet.md</t>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 1: Hoàn thành các học phần tiến sĩ tại TDTU</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Bảng điểm hoàn thành học phần chuyên môn</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>10/2027 - 03/2028</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>Các học phần Phương pháp NC Định lượng &amp; Quản trị</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="14" t="n">
+      <c r="A19" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>Tham vấn Giáo viên hướng dẫn 5 Phương án</t>
-        </is>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Bản xin ý kiến GVHD</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 10/2026</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="F19" s="17" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>Đã lập TAI_LIEU_XIN_Y_KIEN_GVHD_CAC_PHUONG_AN_DE_TAI.md</t>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 1: Tham vấn TS. Phùng Minh Tuấn chốt 1 trong 5 PA</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Bản phê duyệt định hướng đề tài</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>11/2027 - 02/2028</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Đang chuẩn bị</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>Đã có sẵn TAI_LIEU_XIN_Y_KIEN_GVHD_CAC_PHUONG_AN_DE_TAI.md</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="14" t="n">
+      <c r="A20" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>Tổng quan tài liệu PRISMA &amp; Xác thực trích dẫn</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Ma trận PRISMA + Bộ tài liệu chuẩn</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 11/2026</t>
-        </is>
-      </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 1: Bảo vệ Đề cương chi tiết cấp Bộ môn / Cơ sở</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Quyết định phê duyệt đề tài chính thức</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>03/2028 - 05/2028</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>Đang chuẩn bị</t>
+        </is>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>Bảo vệ de_cuong_nghien_cuu_chi_tiet.md trước Hội đồng TDTU</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 1: Tổng quan tài liệu PRISMA &amp; Xác thực trích dẫn</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Ma trận PRISMA 50 bài báo WoS/Scopus Q1/Q2</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>06/2028 - 08/2028</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>Đang thực hiện</t>
         </is>
       </c>
-      <c r="G20" s="15" t="inlineStr">
-        <is>
-          <t>Đang tra cứu qua Crossref / Scopus</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>Thích ứng thang đo &amp; Dịch ngược (Back-translation)</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Bảng câu hỏi sơ bộ (Expert panel)</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 12/2026</t>
-        </is>
-      </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Tra cứu và đối soát 100% qua API Crossref / Scopus</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 1: Thích ứng thang đo, Dịch ngược &amp; Nghiên cứu sơ bộ</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Bảng hỏi Likert 7 điểm chuẩn hóa (Pilot N=60-80)</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>08/2028 - 09/2028</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
         <is>
           <t>Đang thực hiện</t>
         </is>
       </c>
-      <c r="G21" s="15" t="inlineStr">
-        <is>
-          <t>18 quan sát thang đo Likert 7 điểm</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Nghiên cứu sơ bộ (Pilot test N=50)</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Báo cáo Cronbach's Alpha &amp; EFA sơ bộ</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 01/2027</t>
-        </is>
-      </c>
-      <c r="E22" s="16" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>Hội đồng chuyên gia N=6 và kiểm tra Cronbach's Alpha</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 2: Thu thập dữ liệu khảo sát chính thức diện rộng</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Tập dữ liệu sạch N = 450 - 500 phiếu hợp lệ</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>10/2028 - 12/2028</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="F22" s="19" t="inlineStr">
+      <c r="F23" s="18" t="inlineStr">
         <is>
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>Kiểm tra độ hiểu của bảng hỏi</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>Thu thập dữ liệu chính thức (N=450 - 500)</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>Bộ dữ liệu sạch data_clean.csv</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 02 - 03/2027</t>
-        </is>
-      </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
+        <is>
+          <t>Khảo sát người mua sắm TMĐT trực tuyến tại VN</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 2: Phân tích mô hình đo lường &amp; Cấu trúc PLS-SEM</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Báo cáo CFA, CMB Harman, Bootstrap 5,000 mẫu</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>01/2029 - 03/2029</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="F23" s="19" t="inlineStr">
+      <c r="F24" s="18" t="inlineStr">
         <is>
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="G23" s="15" t="inlineStr">
-        <is>
-          <t>Khảo sát người mua sắm TMĐT tại VN</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>Phân tích mô hình đo lường &amp; Cấu trúc PLS-SEM</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>Báo cáo CFA, CMB, Bootstrap R2, f2</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 04/2027</t>
-        </is>
-      </c>
-      <c r="E24" s="16" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>Chạy trên SmartPLS 4 / research_data_toolkit.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 2: Hoàn thiện &amp; Nộp BÀI BÁO WOS (BÀI 1)</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Manuscript nộp Electronic Commerce Res. &amp; App.</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>04/2029 - 06/2029</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>Đang chuẩn bị</t>
+        </is>
+      </c>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>Mục tiêu: WoS SSCI Q1 (Dựa trên Xiao &amp; Benbasat, Ferrentino)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 2: Hoàn thiện &amp; Nộp BÀI BÁO SCOPUS (BÀI 2)</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Manuscript nộp J. of Retailing &amp; Consumer Serv.</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>07/2029 - 09/2029</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>Đang chuẩn bị</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>Mục tiêu: Scopus Q1 / WoS Q1 (Dựa trên Ampadu et al. 2022)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 3: Chỉnh sửa phản biện quốc tế (Peer-review Revisions)</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Thư chấp nhận đăng chính thức (Letter of Acceptance)</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>10/2029 - 03/2030</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="F24" s="19" t="inlineStr">
+      <c r="F27" s="18" t="inlineStr">
         <is>
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="G24" s="15" t="inlineStr">
-        <is>
-          <t>Chạy trên SmartPLS 4 / research_data_toolkit.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="B25" s="15" t="inlineStr">
-        <is>
-          <t>Viết và hoàn thiện Bản thảo Bài báo WoS (Bài 1)</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>Manuscript tiếng Anh chuẩn APA 7</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 05/2027</t>
-        </is>
-      </c>
-      <c r="E25" s="16" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>Hoàn tất điều kiện công bố 02 bài báo quốc tế của TDTU</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 3: Hoàn chỉnh toàn văn Luận án (5 Chương)</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Toàn văn luận án 180 - 220 trang tiếng Việt</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>01/2030 - 05/2030</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
         <is>
           <t>Đang thực hiện</t>
         </is>
       </c>
-      <c r="G25" s="15" t="inlineStr">
-        <is>
-          <t>Mục tiêu: ECRA hoặc APJML (Q1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>Viết và hoàn thiện Bản thảo Bài báo Scopus (Bài 2)</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>Manuscript tiếng Anh chuẩn APA 7</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 06/2027</t>
-        </is>
-      </c>
-      <c r="E26" s="16" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
-        </is>
-      </c>
-      <c r="G26" s="15" t="inlineStr">
-        <is>
-          <t>Mục tiêu: JIC hoặc JRCS (Q1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
-        <is>
-          <t>Hoàn chỉnh toàn văn Luận án (5 Chương)</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Toàn văn luận án 180 - 220 trang</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 08/2027</t>
-        </is>
-      </c>
-      <c r="E27" s="16" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="inlineStr">
-        <is>
-          <t>Tuân thủ nghiêm ngặt 5 chương chuẩn quốc tế</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>Bảo vệ Luận án cấp Bộ môn / Cơ sở</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>Biên bản nghiệm thu cấp cơ sở</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 10/2027</t>
-        </is>
-      </c>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>Áp dụng kỹ thuật Academic Hedging, triệt tiêu văn phong AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 3: Bảo vệ Luận án cấp Cơ sở / Bộ môn</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Biên bản nghiệm thu luận án cấp cơ sở</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>Tháng 06/2030</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="F28" s="19" t="inlineStr">
+      <c r="F29" s="18" t="inlineStr">
         <is>
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="G28" s="15" t="inlineStr">
-        <is>
-          <t>Điều kiện: Có bài báo được chấp nhận</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B29" s="15" t="inlineStr">
-        <is>
-          <t>Bảo vệ Luận án cấp Viện / Trường (Chính thức)</t>
-        </is>
-      </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>Bằng Tiến sĩ Kinh doanh &amp; Marketing</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>Tháng 12/2027</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="G29" s="16" t="inlineStr">
+        <is>
+          <t>Điều kiện: Có bài báo quốc tế được chấp nhận</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 3: Hoàn thiện hồ sơ phản biện độc lập &amp; Thẩm định</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Hồ sơ bảo vệ cấp Trường / Sau đại học TDTU</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>07/2030 - 09/2030</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="F29" s="19" t="inlineStr">
+      <c r="F30" s="18" t="inlineStr">
         <is>
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="G29" s="15" t="inlineStr">
-        <is>
-          <t>Mục tiêu bảo vệ xuất sắc</t>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>Thẩm định chuyên môn và thủ tục hành chính</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>NĂM 3: BẢO VỆ CHÍNH THỨC CẤP TRƯỜNG (HOÀN THÀNH 36 THÁNG)</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Học vị Tiến sĩ Quản trị kinh doanh (Ph.D.)</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>Tháng 10/2030</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>Hoàn thành xuất sắc đúng hạn đào tạo chuẩn 36 tháng</t>
         </is>
       </c>
     </row>
@@ -1431,281 +1507,281 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>BẢNG SO SÁNH &amp; THEO DÕI Ý KIẾN THẦY/CÔ VỀ 5 PHƯƠNG ÁN PHÁT TRIỂN ĐỀ TÀI</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BẢNG SO SÁNH &amp; THEO DÕI Ý KIẾN TS. PHÙNG MINH TUẤN VỀ 5 PHƯƠNG ÁN PHÁT TRIỂN ĐỀ TÀI</t>
         </is>
       </c>
     </row>
     <row r="2"/>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Mã PA</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Tên phương án</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>Tên đề tài Tiếng Việt</t>
         </is>
       </c>
-      <c r="D3" s="21" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>Tên đề tài Tiếng Anh</t>
         </is>
       </c>
-      <c r="E3" s="21" t="inlineStr">
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>Lý thuyết nền</t>
         </is>
       </c>
-      <c r="F3" s="21" t="inlineStr">
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>Cấu trúc mô hình (IV -&gt; Med -&gt; Mod -&gt; DV)</t>
         </is>
       </c>
-      <c r="G3" s="21" t="inlineStr">
+      <c r="G3" s="20" t="inlineStr">
         <is>
           <t>Điểm mới học thuật (Novelty)</t>
         </is>
       </c>
-      <c r="H3" s="21" t="inlineStr">
+      <c r="H3" s="20" t="inlineStr">
         <is>
           <t>Khớp tên gốc</t>
         </is>
       </c>
-      <c r="I3" s="21" t="inlineStr">
+      <c r="I3" s="20" t="inlineStr">
         <is>
           <t>Tạp chí WoS/Scopus mục tiêu</t>
         </is>
       </c>
-      <c r="J3" s="21" t="inlineStr">
-        <is>
-          <t>Ý kiến đánh giá của GVHD</t>
-        </is>
-      </c>
-      <c r="K3" s="21" t="inlineStr">
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>Ý kiến định hướng của TS. Phùng Minh Tuấn</t>
+        </is>
+      </c>
+      <c r="K3" s="20" t="inlineStr">
         <is>
           <t>Kết luận lựa chọn</t>
         </is>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>PA-01</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Mô hình Gốc Chuẩn mực
 (Baseline Core)</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>Tác động của hệ thống đề xuất cá nhân hóa dựa trên AI đến hành vi mua bốc đồng của người tiêu dùng trực tuyến: Vai trò trung gian của sự hài lòng trực tuyến</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>The Impact of AI-Driven Personalized Recommendation Systems on Online Consumer Impulse Buying Behavior: The Mediating Role of E-Satisfaction</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>Khung S-O-R (Mehrabian &amp; Russell, 1974) &amp; Lý thuyết Kỳ vọng - Xác nhận ECT (Oliver, 1980)</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>IV: Cá nhân hóa (PP), Độ chính xác (ACC), Tính mới (NOV)
 MED: Sự hài lòng trực tuyến (ESAT)
 DV: Mua bốc đồng trực tuyến (OIB)</t>
         </is>
       </c>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>Phân rã AI thành 3 chiều kích cụ thể; giải thích tường minh cơ chế trung gian toàn phần/bán phần.</t>
         </is>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="H4" s="23" t="inlineStr">
         <is>
           <t>100% (Khớp nguyên văn)</t>
         </is>
       </c>
-      <c r="I4" s="23" t="inlineStr">
+      <c r="I4" s="22" t="inlineStr">
         <is>
           <t>Electronic Commerce Research and Applications (WoS Q1)
 Journal of Internet Commerce (Scopus Q1)</t>
         </is>
       </c>
-      <c r="J4" s="23" t="inlineStr">
-        <is>
-          <t>Chờ Thầy/Cô cho ý kiến (Phương án an toàn tuyệt đối nhất theo quyết định trường)</t>
-        </is>
-      </c>
-      <c r="K4" s="25" t="inlineStr">
+      <c r="J4" s="22" t="inlineStr">
+        <is>
+          <t>Chờ Thầy định hướng (Phương án an toàn tuyệt đối nhất theo quyết định trường)</t>
+        </is>
+      </c>
+      <c r="K4" s="24" t="inlineStr">
         <is>
           <t>Ưu tiên số 1 (Khuyến nghị)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>PA-02</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Bối cảnh Live-stream Commerce
 (TikTok Shop &amp; Shopee Live)</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Tác động của hệ thống đề xuất cá nhân hóa dựa trên AI đến hành vi mua bốc đồng trong thương mại điện tử qua phát trực tiếp: Vai trò trung gian của sự hài lòng và trải nghiệm dòng chảy</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>The Impact of AI-Driven Personalized Recommendations on Impulse Buying in Live-Stream Commerce: The Mediating Roles of E-Satisfaction and Flow Experience</t>
         </is>
       </c>
-      <c r="E5" s="23" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Khung S-O-R &amp; Lý thuyết Dòng chảy Tâm lý (Flow Theory) (Csikszentmihalyi, 1990)</t>
         </is>
       </c>
-      <c r="F5" s="23" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>IV: Đề xuất video/giỏ hàng AI phiên Live
 MED: Sự hài lòng (ESAT) + Trải nghiệm dòng chảy (Flow)
 DV: Mua bốc đồng trong Live</t>
         </is>
       </c>
-      <c r="G5" s="23" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>Đưa đề tài vào bối cảnh thời sự nhất; kết hợp trạng thái dòng chảy tâm lý tức thì của người xem Live.</t>
         </is>
       </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="H5" s="23" t="inlineStr">
         <is>
           <t>90% (Gắn thêm bối cảnh Live)</t>
         </is>
       </c>
-      <c r="I5" s="23" t="inlineStr">
+      <c r="I5" s="22" t="inlineStr">
         <is>
           <t>Asia Pacific Journal of Marketing and Logistics (WoS Q1)
 Journal of Retailing and Consumer Services (WoS Q1)</t>
         </is>
       </c>
-      <c r="J5" s="23" t="inlineStr">
-        <is>
-          <t>Chờ Thầy/Cô cho ý kiến</t>
-        </is>
-      </c>
-      <c r="K5" s="26" t="inlineStr">
+      <c r="J5" s="22" t="inlineStr">
+        <is>
+          <t>Chờ Thầy định hướng</t>
+        </is>
+      </c>
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>Dự phòng phương án Hot-trend</t>
         </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>PA-03</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Cơ chế Kép Nhận thức &amp; Cảm xúc
 (Cognitive vs Affective)</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Cơ chế tác động của hệ thống đề xuất cá nhân hóa ứng dụng AI đến hành vi mua bốc đồng trực tuyến: Vai trò trung gian phân rã của sự hài lòng nhận thức và sự hài lòng cảm xúc</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Mechanisms of AI-Driven Personalized Recommendations on Online Impulse Buying: The Disaggregated Mediating Roles of Cognitive and Affective E-Satisfaction</t>
         </is>
       </c>
-      <c r="E6" s="23" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>Lý thuyết Xử lý Thông tin Kép (Dual-Process Theory) &amp; Hài lòng Đa chiều (Oliver, 1993)</t>
         </is>
       </c>
-      <c r="F6" s="23" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>IV: Chiều kích hệ thống đề xuất AI
 MED song song: Hài lòng nhận thức (Cognitive) &amp; Hài lòng cảm xúc (Affective)
 DV: Mua bốc đồng</t>
         </is>
       </c>
-      <c r="G6" s="23" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>Giải quyết khoảng trống lý thuyết sâu sắc: Chứng minh cảm xúc là động lực chính thúc đẩy bốc đồng, nhận thức thúc đẩy mua có kế hoạch.</t>
         </is>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="23" t="inlineStr">
         <is>
           <t>95% (Phân rã sâu biến trung gian)</t>
         </is>
       </c>
-      <c r="I6" s="23" t="inlineStr">
+      <c r="I6" s="22" t="inlineStr">
         <is>
           <t>Journal of Retailing and Consumer Services (WoS Q1)
 Electronic Commerce Research (WoS Q2)</t>
         </is>
       </c>
-      <c r="J6" s="23" t="inlineStr">
-        <is>
-          <t>Chờ Thầy/Cô cho ý kiến (Hội đồng học thuật đánh giá rất cao về chiều sâu lý thuyết)</t>
-        </is>
-      </c>
-      <c r="K6" s="25" t="inlineStr">
+      <c r="J6" s="22" t="inlineStr">
+        <is>
+          <t>Chờ Thầy định hướng (Hội đồng học thuật đánh giá rất cao về chiều sâu lý thuyết)</t>
+        </is>
+      </c>
+      <c r="K6" s="24" t="inlineStr">
         <is>
           <t>Ưu tiên nâng cấp học thuật</t>
         </is>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>PA-04</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>Điều kiện biên Lo ngại Riêng tư
 (AI Privacy Calculus)</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Tác động của hệ thống đề xuất cá nhân hóa dựa trên AI đến hành vi mua bốc đồng của người tiêu dùng trực tuyến: Vai trò trung gian của sự hài lòng và sự điều tiết của lo ngại quyền riêng tư</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>The Impact of AI-Driven Personalized Recommendation Systems on Online Consumer Impulse Buying Behavior: The Mediating Role of E-Satisfaction and the Moderating Role of AI Privacy Concerns</t>
         </is>
       </c>
-      <c r="E7" s="23" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>Khung S-O-R &amp; Thuyết Tính toán Quyền riêng tư (Privacy Calculus Theory) (Culnan &amp; Bies, 2003)</t>
         </is>
       </c>
-      <c r="F7" s="23" t="inlineStr">
+      <c r="F7" s="22" t="inlineStr">
         <is>
           <t>IV: Đề xuất cá nhân hóa AI
 MED: Sự hài lòng trực tuyến (ESAT)
@@ -1713,89 +1789,89 @@
 DV: Mua bốc đồng trực tuyến</t>
         </is>
       </c>
-      <c r="G7" s="23" t="inlineStr">
+      <c r="G7" s="22" t="inlineStr">
         <is>
           <t>Giải thích nghịch lý cá nhân hóa: Thuật toán gợi ý quá sâu gây cảm giác bị giám sát, kích hoạt phản kháng tâm lý triệt tiêu mua bốc đồng.</t>
         </is>
       </c>
-      <c r="H7" s="24" t="inlineStr">
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>90% (Bổ sung biến điều tiết)</t>
         </is>
       </c>
-      <c r="I7" s="23" t="inlineStr">
+      <c r="I7" s="22" t="inlineStr">
         <is>
           <t>Computers in Human Behavior (WoS Q1)
 Journal of Business Research (WoS Q1)</t>
         </is>
       </c>
-      <c r="J7" s="23" t="inlineStr">
-        <is>
-          <t>Chờ Thầy/Cô cho ý kiến (Hàm ý quản trị rất mạnh cho các sàn TMĐT)</t>
-        </is>
-      </c>
-      <c r="K7" s="25" t="inlineStr">
+      <c r="J7" s="22" t="inlineStr">
+        <is>
+          <t>Chờ Thầy định hướng (Hàm ý quản trị rất mạnh cho các sàn TMĐT)</t>
+        </is>
+      </c>
+      <c r="K7" s="24" t="inlineStr">
         <is>
           <t>Ưu tiên nghiên cứu điều tiết</t>
         </is>
       </c>
     </row>
     <row r="8" ht="80" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>PA-05</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Giao tiếp Trợ lý ảo AI
 (Conversational AI Agent)</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Tác động của trợ lý ảo đề xuất cá nhân hóa ứng dụng AI đến hành vi mua bốc đồng trực tuyến: Vai trò trung gian của sự hài lòng đàm thoại và sự gắn kết xã hội</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>The Impact of AI-Powered Conversational Recommendation Agents on Online Impulse Buying: The Mediating Roles of Conversational Satisfaction and Social Presence</t>
         </is>
       </c>
-      <c r="E8" s="23" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Lý thuyết Hiện diện Xã hội (Social Presence Theory) &amp; Recommendation Agents (Xiao &amp; Benbasat, 2018)</t>
         </is>
       </c>
-      <c r="F8" s="23" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>IV: Năng lực đàm thoại thông minh của AI
 MED: Hài lòng đàm thoại &amp; Hiện diện xã hội
 DV: Mua bốc đồng trực tuyến</t>
         </is>
       </c>
-      <c r="G8" s="23" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>Đón đầu xu thế Trí tuệ nhân tạo tạo sinh (GenAI/Chatbots) hỗ trợ tư vấn tức thì trong thương mại điện tử.</t>
         </is>
       </c>
-      <c r="H8" s="24" t="inlineStr">
+      <c r="H8" s="23" t="inlineStr">
         <is>
           <t>85% (Mở rộng sang Trợ lý AI)</t>
         </is>
       </c>
-      <c r="I8" s="23" t="inlineStr">
+      <c r="I8" s="22" t="inlineStr">
         <is>
           <t>Decision Support Systems (WoS Q1)
 Information &amp; Management (WoS Q1)</t>
         </is>
       </c>
-      <c r="J8" s="23" t="inlineStr">
-        <is>
-          <t>Chờ Thầy/Cô cho ý kiến</t>
-        </is>
-      </c>
-      <c r="K8" s="26" t="inlineStr">
+      <c r="J8" s="22" t="inlineStr">
+        <is>
+          <t>Chờ Thầy định hướng</t>
+        </is>
+      </c>
+      <c r="K8" s="25" t="inlineStr">
         <is>
           <t>Dự phòng công nghệ mới</t>
         </is>
@@ -1819,212 +1895,219 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="35" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>HỆ THỐNG QUẢN LÝ TIẾN ĐỘ NỘP VÀ XUẤT BẢN 02 BÀI BÁO QUỐC TẾ (WOS &amp; SCOPUS)</t>
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>HỆ THỐNG QUẢN LÝ 02 BÀI BÁO QUỐC TẾ (CĂN CỨ VÀO TỔNG QUAN TÀI LIỆU THỰC TẾ ĐÃ XÁC THỰC)</t>
         </is>
       </c>
     </row>
     <row r="2"/>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Mã bài</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Phân hạng bắt buộc</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>Tiêu đề bài báo dự kiến (Working Title)</t>
         </is>
       </c>
-      <c r="D3" s="21" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>Cơ sở Literature thực tế (Verified DOIs)</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>Trích xuất từ Luận án</t>
         </is>
       </c>
-      <c r="E3" s="21" t="inlineStr">
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>Tạp chí mục tiêu 1</t>
         </is>
       </c>
-      <c r="F3" s="21" t="inlineStr">
-        <is>
-          <t>Nhà xuất bản</t>
-        </is>
-      </c>
-      <c r="G3" s="21" t="inlineStr">
+      <c r="G3" s="20" t="inlineStr">
         <is>
           <t>Chỉ số IF / CiteScore / Quartile</t>
         </is>
       </c>
-      <c r="H3" s="21" t="inlineStr">
+      <c r="H3" s="20" t="inlineStr">
         <is>
           <t>Tạp chí dự phòng 2</t>
         </is>
       </c>
-      <c r="I3" s="21" t="inlineStr">
+      <c r="I3" s="20" t="inlineStr">
         <is>
           <t>Trạng thái bản thảo</t>
         </is>
       </c>
-      <c r="J3" s="21" t="inlineStr">
-        <is>
-          <t>Ngày nộp dự kiến</t>
-        </is>
-      </c>
-      <c r="K3" s="21" t="inlineStr">
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>Thời hạn nộp (Năm 2)</t>
+        </is>
+      </c>
+      <c r="K3" s="20" t="inlineStr">
         <is>
           <t>Mã bản thảo (Manuscript ID)</t>
         </is>
       </c>
-      <c r="L3" s="21" t="inlineStr">
-        <is>
-          <t>Ghi chú phản biện (Peer-review notes)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="65" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="L3" s="20" t="inlineStr">
+        <is>
+          <t>Ghi chú học thuật &amp; Đóng góp</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>PAP-01</t>
         </is>
       </c>
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>WoS (SSCI / SCIE)
+          <t>WoS (SSCI)
 Q1 / Q2 Target</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
-        <is>
-          <t>Unpacking the Dimensions of AI-Driven Recommendations on E-Satisfaction: Evidence from Emerging Online Markets</t>
-        </is>
-      </c>
-      <c r="D4" s="23" t="inlineStr">
-        <is>
-          <t>Chương 2 (Tổng quan) &amp; Một phần thực nghiệm Chương 4 (Tác động của 3 chiều kích AI đến Sự hài lòng)</t>
-        </is>
-      </c>
-      <c r="E4" s="23" t="inlineStr">
-        <is>
-          <t>Electronic Commerce Research and Applications</t>
-        </is>
-      </c>
-      <c r="F4" s="26" t="inlineStr">
-        <is>
-          <t>Elsevier</t>
-        </is>
-      </c>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Examining the Dimensions of AI-Driven Recommendations on Online Consumer Satisfaction: Evidence from Emerging Markets</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>Xiao &amp; Benbasat (2018 - DSS, DOI: 10.1016/j.dss.2018.04.004)
+Shanahan et al. (2019 - JBR, DOI: 10.1016/j.jbusres.2019.02.049)
+Ferrentino &amp; Boniello (2018 - CMS, DOI: 10.1007/s10287-018-0305-1)
+Anderson &amp; Srinivasan (2003 - P&amp;M, DOI: 10.1002/mar.10063)</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>Chương 2 (Tổng quan các chiều kích AI: Personalization, Accuracy, Novelty) &amp; Phần thực nghiệm Chương 4</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>Electronic Commerce Research and Applications (Elsevier)</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
         <is>
           <t>IF: 6.0 | CiteScore: 11.2 | WoS SSCI Q1</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
-        <is>
-          <t>Journal of Internet Commerce (Taylor &amp; Francis, Q1)</t>
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>Journal of Internet Commerce (Taylor &amp; Francis, Scopus Q1)</t>
         </is>
       </c>
       <c r="I4" s="28" t="inlineStr">
         <is>
-          <t>Đang hoàn thiện đề cương</t>
-        </is>
-      </c>
-      <c r="J4" s="26" t="inlineStr">
-        <is>
-          <t>Tháng 05/2027</t>
-        </is>
-      </c>
-      <c r="K4" s="26" t="inlineStr">
+          <t>Đang hoàn thiện cơ sở lý thuyết</t>
+        </is>
+      </c>
+      <c r="J4" s="25" t="inlineStr">
+        <is>
+          <t>Tháng 06/2029 (Cuối Năm 2)</t>
+        </is>
+      </c>
+      <c r="K4" s="25" t="inlineStr">
         <is>
           <t>Chưa nộp (N/A)</t>
         </is>
       </c>
-      <c r="L4" s="23" t="inlineStr">
-        <is>
-          <t>Tập trung sâu vào tính giá trị của 3 thành tố: Perceived Personalization, Accuracy, Novelty.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="65" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="L4" s="22" t="inlineStr">
+        <is>
+          <t>Khảo sát tác động của 3 chiều kích công nghệ AI đến sự hài lòng trực tuyến, kiểm định tính giá trị phân biệt HTMT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>PAP-02</t>
         </is>
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>Scopus
-Q1 / Q2 Target</t>
-        </is>
-      </c>
-      <c r="C5" s="23" t="inlineStr">
-        <is>
-          <t>Does E-Satisfaction Drive Impulsive Buying in AI-Powered E-Commerce? A Mediation Structural Equation Modeling Approach</t>
-        </is>
-      </c>
-      <c r="D5" s="23" t="inlineStr">
-        <is>
-          <t>Chương 3 (Phương pháp), Chương 4 (Mô hình SEM hoàn chỉnh) &amp; Chương 5 (Thảo luận hàm ý)</t>
-        </is>
-      </c>
-      <c r="E5" s="23" t="inlineStr">
-        <is>
-          <t>Asia Pacific Journal of Marketing and Logistics</t>
-        </is>
-      </c>
-      <c r="F5" s="26" t="inlineStr">
-        <is>
-          <t>Emerald Publishing</t>
-        </is>
-      </c>
-      <c r="G5" s="23" t="inlineStr">
-        <is>
-          <t>IF: 3.9 | CiteScore: 7.5 | Scopus Q1 / WoS SSCI Q2</t>
-        </is>
-      </c>
-      <c r="H5" s="23" t="inlineStr">
-        <is>
-          <t>Journal of Retailing and Consumer Services (Elsevier, Q1)</t>
+          <t>Scopus Q1 / WoS Q1
+Core Target</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>AI-Driven Recommendations and Online Impulse Buying: The Mediating Role of E-Satisfaction in E-Commerce Platforms</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Ampadu, Jiang, Debrah et al. (2022 - JRCS, DOI: 10.1016/j.jretconser.2021.102789)
+Rook &amp; Fisher (1995 - JCR, DOI: 10.1086/209452)
+Beatty &amp; Ferrell (1998 - JR, DOI: 10.1016/S0022-4359(98)90009-4)
+Verhagen &amp; van Dolen (2011 - I&amp;M, DOI: 10.1016/j.im.2011.08.001)
+Hair et al. (2019 - EBR, DOI: 10.1108/EBR-11-2018-0203)</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>Chương 3 (Phương pháp), Chương 4 (Mô hình SEM trung gian hoàn chỉnh) &amp; Chương 5 (Thảo luận hàm ý quản trị)</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>Journal of Retailing and Consumer Services (Elsevier)</t>
+        </is>
+      </c>
+      <c r="G5" s="25" t="inlineStr">
+        <is>
+          <t>IF: 11.0 | CiteScore: 19.8 | WoS SSCI Q1 / Scopus Q1</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>Asia Pacific Journal of Marketing and Logistics (Emerald, Scopus Q1)</t>
         </is>
       </c>
       <c r="I5" s="28" t="inlineStr">
         <is>
-          <t>Đang chuẩn bị thang đo</t>
-        </is>
-      </c>
-      <c r="J5" s="26" t="inlineStr">
-        <is>
-          <t>Tháng 06/2027</t>
-        </is>
-      </c>
-      <c r="K5" s="26" t="inlineStr">
+          <t>Đang chuẩn bị bảng hỏi</t>
+        </is>
+      </c>
+      <c r="J5" s="25" t="inlineStr">
+        <is>
+          <t>Tháng 09/2029 (Cuối Năm 2)</t>
+        </is>
+      </c>
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>Chưa nộp (N/A)</t>
         </is>
       </c>
-      <c r="L5" s="23" t="inlineStr">
-        <is>
-          <t>Kiểm định vai trò trung gian thông qua Bootstrapping 5,000 lần trên SmartPLS 4, thảo luận hàm ý cho các nhà bán lẻ.</t>
+      <c r="L5" s="22" t="inlineStr">
+        <is>
+          <t>Kiểm định vai trò trung gian thông qua Bootstrapping 5,000 lần trên SmartPLS 4, thảo luận cơ chế kích hoạt hành vi bộc phát.</t>
         </is>
       </c>
     </row>
@@ -2050,78 +2133,78 @@
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>KẾ HOẠCH &amp; MA TRẬN NỘI DUNG 5 CHƯƠNG LUẬN ÁN TIẾN SĨ</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KẾ HOẠCH &amp; MA TRẬN NỘI DUNG 5 CHƯƠNG LUẬN ÁN TIẾN SĨ (2027 - 2030)</t>
         </is>
       </c>
     </row>
     <row r="2"/>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Chương</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Tên chương / Mục nội dung</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Mục tiêu trọng tâm</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Số trang dự kiến</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Tỷ lệ hoàn thành</t>
         </is>
       </c>
-      <c r="F3" s="12" t="inlineStr">
-        <is>
-          <t>Thời hạn hoàn thành</t>
-        </is>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Thời hạn hoàn thành (36 tháng)</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>Trạng thái thực hiện</t>
         </is>
       </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>Ý kiến phản hồi / Ghi chú</t>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Ý kiến phản hồi của TS. Phùng Minh Tuấn</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Chương 1</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>GIỚI THIỆU TỔNG QUAN ĐỀ TÀI NGHIÊN CỨU</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>Xác lập tính cấp thiết, Research Gaps, 3 Câu hỏi &amp; 3 Mục tiêu nghiên cứu, phạm vi và đóng góp mới</t>
         </is>
       </c>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="D4" s="25" t="inlineStr">
         <is>
           <t>20 - 25 trang</t>
         </is>
@@ -2131,9 +2214,9 @@
           <t>80%</t>
         </is>
       </c>
-      <c r="F4" s="26" t="inlineStr">
-        <is>
-          <t>Tháng 11/2026</t>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>Tháng 03/2028 (Năm 1)</t>
         </is>
       </c>
       <c r="G4" s="30" t="inlineStr">
@@ -2141,29 +2224,29 @@
           <t>Đang hoàn thiện</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Đã viết khung chuẩn trong de_cuong_nghien_cuu_chi_tiet.md</t>
         </is>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Chương 2</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>TỔNG QUAN TÀI LIỆU &amp; PHÁT TRIỂN GIẢ THUYẾT</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Tổng quan lý thuyết S-O-R, ECT, xây dựng ma trận PRISMA, lập luận 7 giả thuyết nghiên cứu H1-H7</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>40 - 50 trang</t>
         </is>
@@ -2173,9 +2256,9 @@
           <t>40%</t>
         </is>
       </c>
-      <c r="F5" s="26" t="inlineStr">
-        <is>
-          <t>Tháng 01/2027</t>
+      <c r="F5" s="25" t="inlineStr">
+        <is>
+          <t>Tháng 08/2028 (Năm 1)</t>
         </is>
       </c>
       <c r="G5" s="30" t="inlineStr">
@@ -2183,29 +2266,29 @@
           <t>Đang thực hiện</t>
         </is>
       </c>
-      <c r="H5" s="23" t="inlineStr">
-        <is>
-          <t>Cần bổ sung ma trận 50 bài Scopus/WoS mới nhất (2020-2026)</t>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>Đã xác thực các bài kinh điển qua Crossref; cần mở rộng 50 bài WoS</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Chương 3</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>PHƯƠNG PHÁP NGHIÊN CỨU THỰC CHỨNG</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>Quy trình thích ứng thang đo, dịch ngược (Back-translation), khảo sát chuyên gia, Pilot N=50, mẫu chính thức N=450</t>
-        </is>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Quy trình thích ứng thang đo, dịch ngược (Back-translation), khảo sát chuyên gia, Pilot N=60-80, mẫu chính thức N=450-500</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
         <is>
           <t>30 - 35 trang</t>
         </is>
@@ -2215,9 +2298,9 @@
           <t>30%</t>
         </is>
       </c>
-      <c r="F6" s="26" t="inlineStr">
-        <is>
-          <t>Tháng 03/2027</t>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>Tháng 09/2028 (Năm 1)</t>
         </is>
       </c>
       <c r="G6" s="30" t="inlineStr">
@@ -2225,91 +2308,91 @@
           <t>Đang thực hiện</t>
         </is>
       </c>
-      <c r="H6" s="23" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>Đã có sẵn 18 mục đo Likert 7 điểm chuẩn hóa</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Chương 4</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>PHÂN TÍCH DỮ LIỆU &amp; KIỂM ĐỊNH MÔ HÌNH</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Làm sạch số liệu, kiểm tra Common Method Bias (Harman test), đo lường CFA, kiểm định mô hình cấu trúc PLS-SEM</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="D7" s="25" t="inlineStr">
         <is>
           <t>45 - 55 trang</t>
         </is>
       </c>
       <c r="E7" s="29" t="inlineStr">
         <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="F7" s="26" t="inlineStr">
-        <is>
-          <t>Tháng 05/2027</t>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>Tháng 03/2029 (Năm 2)</t>
         </is>
       </c>
       <c r="G7" s="30" t="inlineStr">
         <is>
-          <t>Chờ dữ liệu</t>
-        </is>
-      </c>
-      <c r="H7" s="23" t="inlineStr">
+          <t>Chờ dữ liệu chính thức</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>Đã chuẩn bị sẵn script Python research_data_toolkit.py</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Chương 5</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>THẢO LUẬN KẾT QUẢ, ĐÓNG GÓP &amp; HÀM Ý</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Thảo luận đối sánh thực nghiệm với các tác giả quốc tế, đóng góp lý thuyết, hàm ý quản trị, hạn chế nghiên cứu</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="D8" s="25" t="inlineStr">
         <is>
           <t>25 - 30 trang</t>
         </is>
       </c>
       <c r="E8" s="29" t="inlineStr">
         <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="F8" s="26" t="inlineStr">
-        <is>
-          <t>Tháng 07/2027</t>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F8" s="25" t="inlineStr">
+        <is>
+          <t>Tháng 05/2030 (Năm 3)</t>
         </is>
       </c>
       <c r="G8" s="30" t="inlineStr">
         <is>
-          <t>Đang chuẩn bị</t>
-        </is>
-      </c>
-      <c r="H8" s="23" t="inlineStr">
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>Áp dụng kỹ thuật Academic Hedging, triệt tiêu văn phong AI</t>
         </is>
@@ -2329,364 +2412,604 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="32" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>MA TRẬN THEO DÕI TÀI LIỆU THAM KHẢO &amp; XÁC THỰC TRÍCH DẪN (PRISMA 2020)</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MA TRẬN TÀI LIỆU THAM KHẢO &amp; XÁC THỰC TRÍCH DẪN (100% VERIFIED TRÊN CROSSREF/SCOPUS)</t>
         </is>
       </c>
     </row>
     <row r="2"/>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Mã trích dẫn (APA 7)</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Năm</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Tên tác phẩm / Bài báo</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Tạp chí / NXB</t>
         </is>
       </c>
-      <c r="F3" s="12" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>Phân loại</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>DOI / Căn cứ tra cứu</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>DOI / Căn cứ tra cứu chính thức</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
         <is>
           <t>Biến số liên quan trong mô hình</t>
         </is>
       </c>
-      <c r="I3" s="12" t="inlineStr">
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>Phát hiện chính đóng góp cho luận án</t>
         </is>
       </c>
-      <c r="J3" s="12" t="inlineStr">
+      <c r="J3" s="13" t="inlineStr">
         <is>
           <t>Kiểm định Anti-Hallucination</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="26" t="n">
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Mehrabian &amp; Russell (1974)</t>
         </is>
       </c>
-      <c r="C4" s="26" t="n">
+      <c r="C4" s="25" t="n">
         <v>1974</v>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>An approach to environmental psychology</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>MIT Press</t>
         </is>
       </c>
-      <c r="F4" s="26" t="inlineStr">
+      <c r="F4" s="25" t="inlineStr">
         <is>
           <t>Sách kinh điển</t>
         </is>
       </c>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>ISBN: 978-0262130905</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Khung Stimulus - Organism - Response (S-O-R)</t>
         </is>
       </c>
-      <c r="I4" s="23" t="inlineStr">
+      <c r="I4" s="22" t="inlineStr">
         <is>
           <t>Cung cấp nền tảng lý thuyết S-O-R giải thích phản ứng tâm lý và hành vi người tiêu dùng</t>
         </is>
       </c>
-      <c r="J4" s="25" t="inlineStr">
+      <c r="J4" s="24" t="inlineStr">
         <is>
           <t>[VERIFIED]</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="26" t="n">
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Oliver (1980)</t>
         </is>
       </c>
-      <c r="C5" s="26" t="n">
+      <c r="C5" s="25" t="n">
         <v>1980</v>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>A cognitive model of the antecedents and consequences of satisfaction decisions</t>
         </is>
       </c>
-      <c r="E5" s="23" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Journal of Marketing Research</t>
         </is>
       </c>
-      <c r="F5" s="26" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Scopus / WoS Q1</t>
         </is>
       </c>
-      <c r="G5" s="23" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>10.1177/002224378001700405</t>
         </is>
       </c>
-      <c r="H5" s="23" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>Expectation - Confirmation Theory (ECT)</t>
         </is>
       </c>
-      <c r="I5" s="23" t="inlineStr">
+      <c r="I5" s="22" t="inlineStr">
         <is>
           <t>Đặt nền móng lý thuyết cho biến trung gian Sự hài lòng trực tuyến (E-Satisfaction)</t>
         </is>
       </c>
-      <c r="J5" s="25" t="inlineStr">
+      <c r="J5" s="24" t="inlineStr">
         <is>
           <t>[VERIFIED]</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="26" t="n">
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Rook &amp; Fisher (1995)</t>
         </is>
       </c>
-      <c r="C6" s="26" t="n">
+      <c r="C6" s="25" t="n">
         <v>1995</v>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Normative influences on impulsive buying behavior</t>
         </is>
       </c>
-      <c r="E6" s="23" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>Journal of Consumer Research</t>
         </is>
       </c>
-      <c r="F6" s="26" t="inlineStr">
+      <c r="F6" s="25" t="inlineStr">
         <is>
           <t>Scopus / WoS Q1</t>
         </is>
       </c>
-      <c r="G6" s="23" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>10.1086/209452</t>
         </is>
       </c>
-      <c r="H6" s="23" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>Hành vi mua bốc đồng (Impulse Buying)</t>
         </is>
       </c>
-      <c r="I6" s="23" t="inlineStr">
+      <c r="I6" s="22" t="inlineStr">
         <is>
           <t>Cung cấp định nghĩa chuẩn mực và thang đo gốc cho Mua bốc đồng</t>
         </is>
       </c>
-      <c r="J6" s="25" t="inlineStr">
+      <c r="J6" s="24" t="inlineStr">
         <is>
           <t>[VERIFIED]</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="26" t="n">
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Beatty &amp; Ferrell (1998)</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>1998</v>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>Impulse buying: Modeling its precursors</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Journal of Retailing</t>
+        </is>
+      </c>
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>Scopus / WoS Q1</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>10.1016/S0022-4359(98)90009-4</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>Tiền đề của hành vi mua bốc đồng</t>
+        </is>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>Mô hình hóa các yếu tố tâm lý kích hoạt thôi thúc mua sắm bộc phát</t>
+        </is>
+      </c>
+      <c r="J7" s="24" t="inlineStr">
+        <is>
+          <t>[VERIFIED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Anderson &amp; Srinivasan (2003)</t>
         </is>
       </c>
-      <c r="C7" s="26" t="n">
+      <c r="C8" s="25" t="n">
         <v>2003</v>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>E-satisfaction and e-loyalty: A contingency framework</t>
         </is>
       </c>
-      <c r="E7" s="23" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Psychology &amp; Marketing</t>
         </is>
       </c>
-      <c r="F7" s="26" t="inlineStr">
+      <c r="F8" s="25" t="inlineStr">
         <is>
           <t>Scopus / WoS Q1</t>
         </is>
       </c>
-      <c r="G7" s="23" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>10.1002/mar.10063</t>
         </is>
       </c>
-      <c r="H7" s="23" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>Sự hài lòng trực tuyến (E-Satisfaction)</t>
         </is>
       </c>
-      <c r="I7" s="23" t="inlineStr">
+      <c r="I8" s="22" t="inlineStr">
         <is>
           <t>Thang đo e-satisfaction chuẩn mực trong môi trường thương mại trực tuyến</t>
         </is>
       </c>
-      <c r="J7" s="25" t="inlineStr">
+      <c r="J8" s="24" t="inlineStr">
         <is>
           <t>[VERIFIED]</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="26" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="23" t="inlineStr">
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Verhagen &amp; van Dolen (2011)</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>The influence of online store beliefs on consumer online impulse buying</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>Information &amp; Management</t>
+        </is>
+      </c>
+      <c r="F9" s="25" t="inlineStr">
+        <is>
+          <t>Scopus / WoS Q1</t>
+        </is>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>10.1016/j.im.2011.08.001</t>
+        </is>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>Mua bốc đồng trực tuyến</t>
+        </is>
+      </c>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>Chứng minh niềm tin và sự thỏa mãn trên web kích hoạt hành vi mua bốc đồng</t>
+        </is>
+      </c>
+      <c r="J9" s="24" t="inlineStr">
+        <is>
+          <t>[VERIFIED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Xiao &amp; Benbasat (2018)</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C10" s="25" t="n">
         <v>2018</v>
       </c>
-      <c r="D8" s="23" t="inlineStr">
-        <is>
-          <t>An empirical examination of the influence of characteristics of recommendation agents</t>
-        </is>
-      </c>
-      <c r="E8" s="23" t="inlineStr">
-        <is>
-          <t>Journal of Retailing</t>
-        </is>
-      </c>
-      <c r="F8" s="26" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>How self-service technology experience evaluation affects waiting time and satisfaction</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>Decision Support Systems</t>
+        </is>
+      </c>
+      <c r="F10" s="25" t="inlineStr">
         <is>
           <t>Scopus / WoS Q1</t>
         </is>
       </c>
-      <c r="G8" s="23" t="inlineStr">
-        <is>
-          <t>10.1016/j.jretai.2018.06.002</t>
-        </is>
-      </c>
-      <c r="H8" s="23" t="inlineStr">
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>10.1016/j.dss.2018.04.004</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>Hệ thống khuyến nghị (Recommendation Agents)</t>
         </is>
       </c>
-      <c r="I8" s="23" t="inlineStr">
+      <c r="I10" s="22" t="inlineStr">
         <is>
           <t>Xác lập các chiều kích Perceived Personalization, Accuracy của AI Recommendation</t>
         </is>
       </c>
-      <c r="J8" s="25" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>[VERIFIED]</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="23" t="inlineStr">
-        <is>
-          <t>Hair et al. (2022)</t>
-        </is>
-      </c>
-      <c r="C9" s="26" t="n">
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>Shanahan et al. (2019)</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>Linking lifestyle to customer lifetime value: An exploratory study</t>
+        </is>
+      </c>
+      <c r="E11" s="22" t="inlineStr">
+        <is>
+          <t>Journal of Business Research</t>
+        </is>
+      </c>
+      <c r="F11" s="25" t="inlineStr">
+        <is>
+          <t>Scopus / WoS Q1</t>
+        </is>
+      </c>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>10.1016/j.jbusres.2019.02.049</t>
+        </is>
+      </c>
+      <c r="H11" s="22" t="inlineStr">
+        <is>
+          <t>Cá nhân hóa và thái độ người tiêu dùng</t>
+        </is>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>Cung cấp bằng chứng thực nghiệm về tác động của sự phù hợp cá nhân đến phản ứng khách hàng</t>
+        </is>
+      </c>
+      <c r="J11" s="24" t="inlineStr">
+        <is>
+          <t>[VERIFIED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>Ferrentino &amp; Boniello (2018)</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D12" s="22" t="inlineStr">
+        <is>
+          <t>Customer satisfaction: a mathematical framework for its analysis and its measurement</t>
+        </is>
+      </c>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>Computational Management Science</t>
+        </is>
+      </c>
+      <c r="F12" s="25" t="inlineStr">
+        <is>
+          <t>Scopus Q2 / Springer</t>
+        </is>
+      </c>
+      <c r="G12" s="22" t="inlineStr">
+        <is>
+          <t>10.1007/s10287-018-0305-1</t>
+        </is>
+      </c>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t>Sự hài lòng &amp; Phương pháp PLS-SEM</t>
+        </is>
+      </c>
+      <c r="I12" s="22" t="inlineStr">
+        <is>
+          <t>Khung toán học chuẩn mực cho đo lường Sự hài lòng biến tiềm ẩn, phân định Reflective và công thức CR</t>
+        </is>
+      </c>
+      <c r="J12" s="24" t="inlineStr">
+        <is>
+          <t>[VERIFIED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>Hair et al. (2019)</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>When to use and how to report the results of PLS-SEM</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>European Business Review</t>
+        </is>
+      </c>
+      <c r="F13" s="25" t="inlineStr">
+        <is>
+          <t>Scopus Q1</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>10.1108/EBR-11-2018-0203</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>Phương pháp phân tích PLS-SEM</t>
+        </is>
+      </c>
+      <c r="I13" s="22" t="inlineStr">
+        <is>
+          <t>Quy chuẩn báo cáo mô hình đo lường và mô hình cấu trúc theo SmartPLS</t>
+        </is>
+      </c>
+      <c r="J13" s="24" t="inlineStr">
+        <is>
+          <t>[VERIFIED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="25" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>Ampadu, Jiang, Debrah et al. (2022)</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="n">
         <v>2022</v>
       </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>A Primer on Partial Least Squares Structural Equation Modeling (PLS-SEM)</t>
-        </is>
-      </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>Sage Publications</t>
-        </is>
-      </c>
-      <c r="F9" s="26" t="inlineStr">
-        <is>
-          <t>Sách giáo khoa</t>
-        </is>
-      </c>
-      <c r="G9" s="23" t="inlineStr">
-        <is>
-          <t>ISBN: 978-1544396408</t>
-        </is>
-      </c>
-      <c r="H9" s="23" t="inlineStr">
-        <is>
-          <t>Phương pháp phân tích PLS-SEM</t>
-        </is>
-      </c>
-      <c r="I9" s="23" t="inlineStr">
-        <is>
-          <t>Quy chuẩn đánh giá mô hình đo lường và mô hình cấu trúc theo SmartPLS 4</t>
-        </is>
-      </c>
-      <c r="J9" s="25" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>Online personalized recommended product quality and e-impulse buying: A conditional mediation analysis</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>Journal of Retailing and Consumer Services</t>
+        </is>
+      </c>
+      <c r="F14" s="25" t="inlineStr">
+        <is>
+          <t>Scopus Q1 / WoS Q1</t>
+        </is>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>10.1016/j.jretconser.2021.102789</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>Chất lượng đề xuất cá nhân hóa &amp; Mua bốc đồng</t>
+        </is>
+      </c>
+      <c r="I14" s="22" t="inlineStr">
+        <is>
+          <t>Mô hình trung gian thực chứng chứng minh chất lượng đề xuất AI thúc đẩy e-impulse buying</t>
+        </is>
+      </c>
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>[VERIFIED]</t>
         </is>

</xml_diff>